<commit_message>
Ran through EDM analysis with and without various corrections, and verified correction in sim again
</commit_message>
<xml_diff>
--- a/Sheets/VerticalOffsetSlopes.xlsx
+++ b/Sheets/VerticalOffsetSlopes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A64D32B1-863B-5944-8066-E01D8BDE6807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F9CCBA7-15CB-2F43-8042-76EEFCB79B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2120" yWindow="-20220" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{46C0C8EE-F9CC-6B4A-9F1A-AF04040EA546}"/>
+    <workbookView xWindow="0" yWindow="520" windowWidth="28800" windowHeight="17500" xr2:uid="{46C0C8EE-F9CC-6B4A-9F1A-AF04040EA546}"/>
   </bookViews>
   <sheets>
     <sheet name="draft" sheetId="1" r:id="rId1"/>
@@ -3510,13 +3510,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:ln w="25400" cap="rnd">
-                <a:noFill/>
-                <a:round/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-D449-0B41-9EE6-92592D6B02F3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:trendline>
             <c:spPr>
@@ -3719,13 +3717,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:ln w="25400" cap="rnd">
-                <a:noFill/>
-                <a:round/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-D449-0B41-9EE6-92592D6B02F3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:trendline>
             <c:spPr>
@@ -3938,13 +3934,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:ln w="25400" cap="rnd">
-                <a:noFill/>
-                <a:round/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-D449-0B41-9EE6-92592D6B02F3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:errBars>
             <c:errDir val="x"/>
@@ -4090,6 +4084,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000008-D449-0B41-9EE6-92592D6B02F3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:errBars>
             <c:errDir val="x"/>
@@ -6834,6 +6833,37 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>

</xml_diff>